<commit_message>
update prop book & edit cumulative view on 3_Historical
</commit_message>
<xml_diff>
--- a/sql/Prop book.xlsx
+++ b/sql/Prop book.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Thao Dien\Broker-page - Copy\sql\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4567CC0A-2E50-45C3-A8BA-4541552761D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4437B17-C19C-495F-B0EC-7544AE38DBB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="795" yWindow="675" windowWidth="25200" windowHeight="14505" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$320</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$326</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="980" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="998" uniqueCount="92">
   <si>
     <t>Broker</t>
   </si>
@@ -309,6 +309,9 @@
   </si>
   <si>
     <t>SAB</t>
+  </si>
+  <si>
+    <t>REE</t>
   </si>
 </sst>
 </file>
@@ -672,14 +675,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:E326"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:E332"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="5" max="6" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -696,7 +698,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -710,7 +712,7 @@
         <v>598.5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -724,7 +726,7 @@
         <v>81.7</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -738,7 +740,7 @@
         <v>1945.2</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -749,7 +751,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -763,7 +765,7 @@
         <v>180.69</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -777,7 +779,7 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -791,7 +793,7 @@
         <v>232.999</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -805,7 +807,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -819,7 +821,7 @@
         <v>2756</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -833,7 +835,7 @@
         <v>796.99</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>5</v>
       </c>
@@ -844,7 +846,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -858,7 +860,7 @@
         <v>1882.8</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>5</v>
       </c>
@@ -872,7 +874,7 @@
         <v>11.73</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>5</v>
       </c>
@@ -886,7 +888,7 @@
         <v>297.25</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>5</v>
       </c>
@@ -900,7 +902,7 @@
         <v>139.4</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>5</v>
       </c>
@@ -914,7 +916,7 @@
         <v>803.12</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>5</v>
       </c>
@@ -928,7 +930,7 @@
         <v>837.54</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>5</v>
       </c>
@@ -942,7 +944,7 @@
         <v>1673.2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>5</v>
       </c>
@@ -956,7 +958,7 @@
         <v>1184</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>5</v>
       </c>
@@ -967,7 +969,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>5</v>
       </c>
@@ -981,7 +983,7 @@
         <v>2117.6</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>5</v>
       </c>
@@ -992,7 +994,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>5</v>
       </c>
@@ -1006,7 +1008,7 @@
         <v>12.33</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>5</v>
       </c>
@@ -1020,7 +1022,7 @@
         <v>167.5</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>5</v>
       </c>
@@ -1034,7 +1036,7 @@
         <v>695.36</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>5</v>
       </c>
@@ -1048,7 +1050,7 @@
         <v>772.4</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>5</v>
       </c>
@@ -1062,7 +1064,7 @@
         <v>2070</v>
       </c>
     </row>
-    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>18</v>
       </c>
@@ -1076,7 +1078,7 @@
         <v>172.64</v>
       </c>
     </row>
-    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>18</v>
       </c>
@@ -1090,7 +1092,7 @@
         <v>282.2</v>
       </c>
     </row>
-    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>18</v>
       </c>
@@ -1104,7 +1106,7 @@
         <v>7.84</v>
       </c>
     </row>
-    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>18</v>
       </c>
@@ -1118,7 +1120,7 @@
         <v>64.372</v>
       </c>
     </row>
-    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>18</v>
       </c>
@@ -1132,7 +1134,7 @@
         <v>105.5</v>
       </c>
     </row>
-    <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>18</v>
       </c>
@@ -1146,7 +1148,7 @@
         <v>87.8</v>
       </c>
     </row>
-    <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>18</v>
       </c>
@@ -1160,7 +1162,7 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>26</v>
       </c>
@@ -1174,7 +1176,7 @@
         <v>287.54000000000002</v>
       </c>
     </row>
-    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>26</v>
       </c>
@@ -1188,7 +1190,7 @@
         <v>177.85</v>
       </c>
     </row>
-    <row r="38" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>26</v>
       </c>
@@ -1202,7 +1204,7 @@
         <v>252.98500000000001</v>
       </c>
     </row>
-    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>26</v>
       </c>
@@ -1216,7 +1218,7 @@
         <v>91.463300000000004</v>
       </c>
     </row>
-    <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>26</v>
       </c>
@@ -1227,7 +1229,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>26</v>
       </c>
@@ -1242,7 +1244,7 @@
         <v>3843.058</v>
       </c>
     </row>
-    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>26</v>
       </c>
@@ -1256,7 +1258,7 @@
         <v>275.23899999999998</v>
       </c>
     </row>
-    <row r="43" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>26</v>
       </c>
@@ -1270,7 +1272,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>18</v>
       </c>
@@ -1284,7 +1286,7 @@
         <v>189.8</v>
       </c>
     </row>
-    <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>18</v>
       </c>
@@ -1298,7 +1300,7 @@
         <v>106.4</v>
       </c>
     </row>
-    <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>18</v>
       </c>
@@ -1312,7 +1314,7 @@
         <v>204.8</v>
       </c>
     </row>
-    <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>18</v>
       </c>
@@ -1326,7 +1328,7 @@
         <v>79.099999999999994</v>
       </c>
     </row>
-    <row r="48" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>18</v>
       </c>
@@ -1340,7 +1342,7 @@
         <v>70.599999999999994</v>
       </c>
     </row>
-    <row r="49" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>18</v>
       </c>
@@ -1354,7 +1356,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="50" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>18</v>
       </c>
@@ -1368,7 +1370,7 @@
         <v>170.9</v>
       </c>
     </row>
-    <row r="51" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>18</v>
       </c>
@@ -1382,7 +1384,7 @@
         <v>238.4</v>
       </c>
     </row>
-    <row r="52" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>18</v>
       </c>
@@ -1396,7 +1398,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="53" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>18</v>
       </c>
@@ -1410,7 +1412,7 @@
         <v>91.6</v>
       </c>
     </row>
-    <row r="54" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>18</v>
       </c>
@@ -1424,7 +1426,7 @@
         <v>71.3</v>
       </c>
     </row>
-    <row r="55" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>18</v>
       </c>
@@ -1438,7 +1440,7 @@
         <v>47.6</v>
       </c>
     </row>
-    <row r="56" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>18</v>
       </c>
@@ -1452,7 +1454,7 @@
         <v>178.9</v>
       </c>
     </row>
-    <row r="57" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>18</v>
       </c>
@@ -1466,7 +1468,7 @@
         <v>10.3</v>
       </c>
     </row>
-    <row r="58" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>23</v>
       </c>
@@ -1480,7 +1482,7 @@
         <v>1635</v>
       </c>
     </row>
-    <row r="59" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>23</v>
       </c>
@@ -1494,7 +1496,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="60" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>23</v>
       </c>
@@ -1508,7 +1510,7 @@
         <v>734.97</v>
       </c>
     </row>
-    <row r="61" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>23</v>
       </c>
@@ -1522,7 +1524,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>23</v>
       </c>
@@ -1536,7 +1538,7 @@
         <v>683.3</v>
       </c>
     </row>
-    <row r="63" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>23</v>
       </c>
@@ -1550,7 +1552,7 @@
         <v>428.9</v>
       </c>
     </row>
-    <row r="64" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>23</v>
       </c>
@@ -1564,7 +1566,7 @@
         <v>4362.4489999999996</v>
       </c>
     </row>
-    <row r="65" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>23</v>
       </c>
@@ -1578,7 +1580,7 @@
         <v>684.67200000000003</v>
       </c>
     </row>
-    <row r="66" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>23</v>
       </c>
@@ -1592,7 +1594,7 @@
         <v>873</v>
       </c>
     </row>
-    <row r="67" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>23</v>
       </c>
@@ -1606,7 +1608,7 @@
         <v>298.214</v>
       </c>
     </row>
-    <row r="68" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>26</v>
       </c>
@@ -1620,7 +1622,7 @@
         <v>462.96722006800002</v>
       </c>
     </row>
-    <row r="69" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>23</v>
       </c>
@@ -1634,7 +1636,7 @@
         <v>1602.507328938</v>
       </c>
     </row>
-    <row r="70" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>26</v>
       </c>
@@ -1648,7 +1650,7 @@
         <v>281.90273591300001</v>
       </c>
     </row>
-    <row r="71" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>26</v>
       </c>
@@ -1662,7 +1664,7 @@
         <v>325.68608381000001</v>
       </c>
     </row>
-    <row r="72" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>23</v>
       </c>
@@ -1676,7 +1678,7 @@
         <v>133.6666776649999</v>
       </c>
     </row>
-    <row r="73" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>23</v>
       </c>
@@ -1690,7 +1692,7 @@
         <v>465.20486131000013</v>
       </c>
     </row>
-    <row r="74" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>18</v>
       </c>
@@ -1704,7 +1706,7 @@
         <v>73.276574532000055</v>
       </c>
     </row>
-    <row r="75" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>18</v>
       </c>
@@ -1718,7 +1720,7 @@
         <v>132.5779621770001</v>
       </c>
     </row>
-    <row r="76" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>18</v>
       </c>
@@ -1732,7 +1734,7 @@
         <v>217.38459526099999</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>5</v>
       </c>
@@ -1746,7 +1748,7 @@
         <v>253.33511597899991</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>5</v>
       </c>
@@ -1760,7 +1762,7 @@
         <v>355.10702067800003</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>5</v>
       </c>
@@ -1774,7 +1776,7 @@
         <v>211.49055106</v>
       </c>
     </row>
-    <row r="80" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>26</v>
       </c>
@@ -1788,7 +1790,7 @@
         <v>313.72500000000002</v>
       </c>
     </row>
-    <row r="81" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>26</v>
       </c>
@@ -1802,7 +1804,7 @@
         <v>252.69882000000001</v>
       </c>
     </row>
-    <row r="82" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>26</v>
       </c>
@@ -1816,7 +1818,7 @@
         <v>131.61000000000001</v>
       </c>
     </row>
-    <row r="83" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>26</v>
       </c>
@@ -1830,7 +1832,7 @@
         <v>115.5</v>
       </c>
     </row>
-    <row r="84" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>26</v>
       </c>
@@ -1844,7 +1846,7 @@
         <v>80.653409999999994</v>
       </c>
     </row>
-    <row r="85" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>26</v>
       </c>
@@ -1858,7 +1860,7 @@
         <v>4593.8958050000001</v>
       </c>
     </row>
-    <row r="86" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>26</v>
       </c>
@@ -1869,7 +1871,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="87" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>26</v>
       </c>
@@ -1880,7 +1882,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="88" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>26</v>
       </c>
@@ -1894,7 +1896,7 @@
         <v>385.00864000000001</v>
       </c>
     </row>
-    <row r="89" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>26</v>
       </c>
@@ -1908,7 +1910,7 @@
         <v>204.87155000000001</v>
       </c>
     </row>
-    <row r="90" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>26</v>
       </c>
@@ -1922,7 +1924,7 @@
         <v>449.16890000000001</v>
       </c>
     </row>
-    <row r="91" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>26</v>
       </c>
@@ -1936,7 +1938,7 @@
         <v>298.416</v>
       </c>
     </row>
-    <row r="92" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>26</v>
       </c>
@@ -1950,7 +1952,7 @@
         <v>2868.1795425969999</v>
       </c>
     </row>
-    <row r="93" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>26</v>
       </c>
@@ -1961,7 +1963,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="94" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>26</v>
       </c>
@@ -1972,7 +1974,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="95" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>44</v>
       </c>
@@ -1986,7 +1988,7 @@
         <v>471.11800299999999</v>
       </c>
     </row>
-    <row r="96" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>44</v>
       </c>
@@ -2000,7 +2002,7 @@
         <v>444.90018559999999</v>
       </c>
     </row>
-    <row r="97" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>44</v>
       </c>
@@ -2014,7 +2016,7 @@
         <v>194.95070833</v>
       </c>
     </row>
-    <row r="98" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>44</v>
       </c>
@@ -2028,7 +2030,7 @@
         <v>459.73992199999998</v>
       </c>
     </row>
-    <row r="99" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>44</v>
       </c>
@@ -2042,7 +2044,7 @@
         <v>105.4291377</v>
       </c>
     </row>
-    <row r="100" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>44</v>
       </c>
@@ -2056,7 +2058,7 @@
         <v>112.9934461</v>
       </c>
     </row>
-    <row r="101" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>44</v>
       </c>
@@ -2070,7 +2072,7 @@
         <v>795.19149128900006</v>
       </c>
     </row>
-    <row r="102" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>44</v>
       </c>
@@ -2084,7 +2086,7 @@
         <v>418.20360959999999</v>
       </c>
     </row>
-    <row r="103" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>44</v>
       </c>
@@ -2098,7 +2100,7 @@
         <v>379.16809019999999</v>
       </c>
     </row>
-    <row r="104" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>44</v>
       </c>
@@ -2112,7 +2114,7 @@
         <v>641.44849673199997</v>
       </c>
     </row>
-    <row r="105" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>46</v>
       </c>
@@ -2126,7 +2128,7 @@
         <v>495.18126749999999</v>
       </c>
     </row>
-    <row r="106" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>46</v>
       </c>
@@ -2140,7 +2142,7 @@
         <v>41.564160000000001</v>
       </c>
     </row>
-    <row r="107" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>46</v>
       </c>
@@ -2154,7 +2156,7 @@
         <v>34.574301900000002</v>
       </c>
     </row>
-    <row r="108" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>46</v>
       </c>
@@ -2168,7 +2170,7 @@
         <v>17.764817699999998</v>
       </c>
     </row>
-    <row r="109" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>46</v>
       </c>
@@ -2182,7 +2184,7 @@
         <v>377.74047731399997</v>
       </c>
     </row>
-    <row r="110" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>46</v>
       </c>
@@ -2196,7 +2198,7 @@
         <v>47.814399999999999</v>
       </c>
     </row>
-    <row r="111" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>46</v>
       </c>
@@ -2210,7 +2212,7 @@
         <v>105.3778854</v>
       </c>
     </row>
-    <row r="112" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>46</v>
       </c>
@@ -2224,7 +2226,7 @@
         <v>45.304979000000003</v>
       </c>
     </row>
-    <row r="113" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>46</v>
       </c>
@@ -2238,7 +2240,7 @@
         <v>883.491355</v>
       </c>
     </row>
-    <row r="114" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>46</v>
       </c>
@@ -2252,7 +2254,7 @@
         <v>329.83531951999998</v>
       </c>
     </row>
-    <row r="115" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>46</v>
       </c>
@@ -2266,7 +2268,7 @@
         <v>56.4498575</v>
       </c>
     </row>
-    <row r="116" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>46</v>
       </c>
@@ -2280,7 +2282,7 @@
         <v>48.783651149999997</v>
       </c>
     </row>
-    <row r="117" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>46</v>
       </c>
@@ -2294,7 +2296,7 @@
         <v>53.905700000000003</v>
       </c>
     </row>
-    <row r="118" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>46</v>
       </c>
@@ -2308,7 +2310,7 @@
         <v>897.44555519999994</v>
       </c>
     </row>
-    <row r="119" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>46</v>
       </c>
@@ -2322,7 +2324,7 @@
         <v>567.41111581400003</v>
       </c>
     </row>
-    <row r="120" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>50</v>
       </c>
@@ -2336,7 +2338,7 @@
         <v>1219.89348</v>
       </c>
     </row>
-    <row r="121" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>50</v>
       </c>
@@ -2350,7 +2352,7 @@
         <v>891.07434000000001</v>
       </c>
     </row>
-    <row r="122" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>50</v>
       </c>
@@ -2364,7 +2366,7 @@
         <v>386.46965</v>
       </c>
     </row>
-    <row r="123" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>50</v>
       </c>
@@ -2378,7 +2380,7 @@
         <v>376.3553</v>
       </c>
     </row>
-    <row r="124" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>50</v>
       </c>
@@ -2392,7 +2394,7 @@
         <v>258.97612800000002</v>
       </c>
     </row>
-    <row r="125" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>50</v>
       </c>
@@ -2406,7 +2408,7 @@
         <v>157.063692</v>
       </c>
     </row>
-    <row r="126" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>50</v>
       </c>
@@ -2420,7 +2422,7 @@
         <v>80.896979999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>50</v>
       </c>
@@ -2434,7 +2436,7 @@
         <v>66.592600000000004</v>
       </c>
     </row>
-    <row r="128" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>50</v>
       </c>
@@ -2448,7 +2450,7 @@
         <v>35.567970000000003</v>
       </c>
     </row>
-    <row r="129" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>50</v>
       </c>
@@ -2462,7 +2464,7 @@
         <v>32.722560000000001</v>
       </c>
     </row>
-    <row r="130" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>50</v>
       </c>
@@ -2476,7 +2478,7 @@
         <v>76.413469636000002</v>
       </c>
     </row>
-    <row r="131" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>50</v>
       </c>
@@ -2490,7 +2492,7 @@
         <v>51.984900000000003</v>
       </c>
     </row>
-    <row r="132" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>50</v>
       </c>
@@ -2504,7 +2506,7 @@
         <v>54.700949999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>50</v>
       </c>
@@ -2518,7 +2520,7 @@
         <v>43.162300000000002</v>
       </c>
     </row>
-    <row r="134" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>50</v>
       </c>
@@ -2532,7 +2534,7 @@
         <v>37.572000000000003</v>
       </c>
     </row>
-    <row r="135" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>50</v>
       </c>
@@ -2546,7 +2548,7 @@
         <v>26.318750000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>50</v>
       </c>
@@ -2560,7 +2562,7 @@
         <v>24.028199999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>50</v>
       </c>
@@ -2574,7 +2576,7 @@
         <v>21.36645</v>
       </c>
     </row>
-    <row r="138" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>50</v>
       </c>
@@ -2588,7 +2590,7 @@
         <v>17.355250000000002</v>
       </c>
     </row>
-    <row r="139" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>50</v>
       </c>
@@ -2602,7 +2604,7 @@
         <v>17.120100000000001</v>
       </c>
     </row>
-    <row r="140" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>50</v>
       </c>
@@ -2616,7 +2618,7 @@
         <v>16.202475</v>
       </c>
     </row>
-    <row r="141" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>50</v>
       </c>
@@ -2630,7 +2632,7 @@
         <v>13.5169</v>
       </c>
     </row>
-    <row r="142" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>50</v>
       </c>
@@ -2644,7 +2646,7 @@
         <v>8.3619000000000003</v>
       </c>
     </row>
-    <row r="143" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>50</v>
       </c>
@@ -2658,7 +2660,7 @@
         <v>2.3957999999999999</v>
       </c>
     </row>
-    <row r="144" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>50</v>
       </c>
@@ -2672,7 +2674,7 @@
         <v>1791.136023734</v>
       </c>
     </row>
-    <row r="145" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>50</v>
       </c>
@@ -2686,7 +2688,7 @@
         <v>691.42874749999999</v>
       </c>
     </row>
-    <row r="146" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>50</v>
       </c>
@@ -2700,7 +2702,7 @@
         <v>437.546178</v>
       </c>
     </row>
-    <row r="147" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>50</v>
       </c>
@@ -2714,7 +2716,7 @@
         <v>398.44944659999999</v>
       </c>
     </row>
-    <row r="148" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>50</v>
       </c>
@@ -2728,7 +2730,7 @@
         <v>85.158848000000006</v>
       </c>
     </row>
-    <row r="149" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>50</v>
       </c>
@@ -2742,7 +2744,7 @@
         <v>56.339108600000003</v>
       </c>
     </row>
-    <row r="150" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>50</v>
       </c>
@@ -2756,7 +2758,7 @@
         <v>50.207640599999998</v>
       </c>
     </row>
-    <row r="151" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>50</v>
       </c>
@@ -2770,7 +2772,7 @@
         <v>48.181075200000002</v>
       </c>
     </row>
-    <row r="152" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>50</v>
       </c>
@@ -2784,7 +2786,7 @@
         <v>48.151496999999999</v>
       </c>
     </row>
-    <row r="153" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>50</v>
       </c>
@@ -2798,7 +2800,7 @@
         <v>38.785400000000003</v>
       </c>
     </row>
-    <row r="154" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>50</v>
       </c>
@@ -2812,7 +2814,7 @@
         <v>33.768990000000002</v>
       </c>
     </row>
-    <row r="155" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>50</v>
       </c>
@@ -2826,7 +2828,7 @@
         <v>27.742000000000001</v>
       </c>
     </row>
-    <row r="156" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>50</v>
       </c>
@@ -2840,7 +2842,7 @@
         <v>26.166374399999999</v>
       </c>
     </row>
-    <row r="157" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>50</v>
       </c>
@@ -2854,7 +2856,7 @@
         <v>312.90250348900003</v>
       </c>
     </row>
-    <row r="158" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>61</v>
       </c>
@@ -2868,7 +2870,7 @@
         <v>537.23077231399998</v>
       </c>
     </row>
-    <row r="159" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>61</v>
       </c>
@@ -2882,7 +2884,7 @@
         <v>1.2738610640000001</v>
       </c>
     </row>
-    <row r="160" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>61</v>
       </c>
@@ -2896,7 +2898,7 @@
         <v>571.68737199999998</v>
       </c>
     </row>
-    <row r="161" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>61</v>
       </c>
@@ -2910,7 +2912,7 @@
         <v>1.2426057850000001</v>
       </c>
     </row>
-    <row r="162" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>63</v>
       </c>
@@ -2924,7 +2926,7 @@
         <v>81.770314499999998</v>
       </c>
     </row>
-    <row r="163" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>63</v>
       </c>
@@ -2938,7 +2940,7 @@
         <v>114.13664420000001</v>
       </c>
     </row>
-    <row r="164" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>63</v>
       </c>
@@ -2952,7 +2954,7 @@
         <v>74.028000000000006</v>
       </c>
     </row>
-    <row r="165" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>63</v>
       </c>
@@ -2966,7 +2968,7 @@
         <v>334.50573044999999</v>
       </c>
     </row>
-    <row r="166" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>63</v>
       </c>
@@ -2980,7 +2982,7 @@
         <v>82.876750000000001</v>
       </c>
     </row>
-    <row r="167" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>63</v>
       </c>
@@ -2994,7 +2996,7 @@
         <v>96.033543249999994</v>
       </c>
     </row>
-    <row r="168" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>63</v>
       </c>
@@ -3008,7 +3010,7 @@
         <v>619.63735652000003</v>
       </c>
     </row>
-    <row r="169" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>63</v>
       </c>
@@ -3022,7 +3024,7 @@
         <v>66.806430000000006</v>
       </c>
     </row>
-    <row r="170" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>63</v>
       </c>
@@ -3036,7 +3038,7 @@
         <v>62.841739349999997</v>
       </c>
     </row>
-    <row r="171" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>63</v>
       </c>
@@ -3050,7 +3052,7 @@
         <v>64.178100000000001</v>
       </c>
     </row>
-    <row r="172" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>63</v>
       </c>
@@ -3064,7 +3066,7 @@
         <v>462.98242733000001</v>
       </c>
     </row>
-    <row r="173" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>64</v>
       </c>
@@ -3075,7 +3077,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="174" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>64</v>
       </c>
@@ -3089,7 +3091,7 @@
         <v>1.0325E-4</v>
       </c>
     </row>
-    <row r="175" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>64</v>
       </c>
@@ -3100,7 +3102,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="176" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>64</v>
       </c>
@@ -3114,7 +3116,7 @@
         <v>1.1900000000000001E-4</v>
       </c>
     </row>
-    <row r="177" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>64</v>
       </c>
@@ -3125,7 +3127,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="178" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>67</v>
       </c>
@@ -3139,7 +3141,7 @@
         <v>64.729280000000003</v>
       </c>
     </row>
-    <row r="179" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>67</v>
       </c>
@@ -3153,7 +3155,7 @@
         <v>4.1003119999999997</v>
       </c>
     </row>
-    <row r="180" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>67</v>
       </c>
@@ -3167,7 +3169,7 @@
         <v>7.8800173759999996</v>
       </c>
     </row>
-    <row r="181" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>67</v>
       </c>
@@ -3181,7 +3183,7 @@
         <v>57.4816</v>
       </c>
     </row>
-    <row r="182" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>67</v>
       </c>
@@ -3195,7 +3197,7 @@
         <v>3.4080650000000001E-3</v>
       </c>
     </row>
-    <row r="183" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>67</v>
       </c>
@@ -3209,7 +3211,7 @@
         <v>9.5435766019999999</v>
       </c>
     </row>
-    <row r="184" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>67</v>
       </c>
@@ -3223,7 +3225,7 @@
         <v>3.4080650000000001E-3</v>
       </c>
     </row>
-    <row r="185" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>63</v>
       </c>
@@ -3237,7 +3239,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="186" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>63</v>
       </c>
@@ -3251,7 +3253,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="187" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>63</v>
       </c>
@@ -3265,7 +3267,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="188" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>61</v>
       </c>
@@ -3279,7 +3281,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="189" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>61</v>
       </c>
@@ -3293,7 +3295,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="190" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>61</v>
       </c>
@@ -3307,7 +3309,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="191" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>50</v>
       </c>
@@ -3321,7 +3323,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="192" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>50</v>
       </c>
@@ -3335,7 +3337,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="193" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>50</v>
       </c>
@@ -3349,7 +3351,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="194" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>64</v>
       </c>
@@ -3363,7 +3365,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="195" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>64</v>
       </c>
@@ -3377,7 +3379,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="196" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>64</v>
       </c>
@@ -3391,7 +3393,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="197" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>67</v>
       </c>
@@ -3405,7 +3407,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="198" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>67</v>
       </c>
@@ -3419,7 +3421,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="199" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>67</v>
       </c>
@@ -3433,7 +3435,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="200" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>26</v>
       </c>
@@ -3447,7 +3449,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="201" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>26</v>
       </c>
@@ -3461,7 +3463,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="202" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>26</v>
       </c>
@@ -3475,7 +3477,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="203" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>46</v>
       </c>
@@ -3489,7 +3491,7 @@
         <v>1198</v>
       </c>
     </row>
-    <row r="204" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>46</v>
       </c>
@@ -3503,7 +3505,7 @@
         <v>1047</v>
       </c>
     </row>
-    <row r="205" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>46</v>
       </c>
@@ -3517,7 +3519,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="206" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>44</v>
       </c>
@@ -3531,7 +3533,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="207" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>44</v>
       </c>
@@ -3545,7 +3547,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="208" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>44</v>
       </c>
@@ -3559,7 +3561,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="209" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>70</v>
       </c>
@@ -3573,7 +3575,7 @@
         <v>291.53755000000001</v>
       </c>
     </row>
-    <row r="210" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
         <v>70</v>
       </c>
@@ -3587,7 +3589,7 @@
         <v>97.599699999999999</v>
       </c>
     </row>
-    <row r="211" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
         <v>70</v>
       </c>
@@ -3601,7 +3603,7 @@
         <v>139.96039999999999</v>
       </c>
     </row>
-    <row r="212" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
         <v>70</v>
       </c>
@@ -3615,7 +3617,7 @@
         <v>126.0891627</v>
       </c>
     </row>
-    <row r="213" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
         <v>70</v>
       </c>
@@ -3629,7 +3631,7 @@
         <v>484.16045324999999</v>
       </c>
     </row>
-    <row r="214" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
         <v>70</v>
       </c>
@@ -3643,7 +3645,7 @@
         <v>97.860349999999997</v>
       </c>
     </row>
-    <row r="215" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>70</v>
       </c>
@@ -3657,7 +3659,7 @@
         <v>118.3644</v>
       </c>
     </row>
-    <row r="216" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
         <v>70</v>
       </c>
@@ -3671,7 +3673,7 @@
         <v>40.125</v>
       </c>
     </row>
-    <row r="217" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
         <v>70</v>
       </c>
@@ -3685,7 +3687,7 @@
         <v>-17.442687286000002</v>
       </c>
     </row>
-    <row r="218" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
         <v>70</v>
       </c>
@@ -3699,7 +3701,7 @@
         <v>319.48334</v>
       </c>
     </row>
-    <row r="219" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
         <v>70</v>
       </c>
@@ -3713,7 +3715,7 @@
         <v>1110.0100874</v>
       </c>
     </row>
-    <row r="220" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
         <v>70</v>
       </c>
@@ -3727,7 +3729,7 @@
         <v>131.24760000000001</v>
       </c>
     </row>
-    <row r="221" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>70</v>
       </c>
@@ -3741,7 +3743,7 @@
         <v>77.801199999999994</v>
       </c>
     </row>
-    <row r="222" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
         <v>70</v>
       </c>
@@ -3755,7 +3757,7 @@
         <v>49.610999999999997</v>
       </c>
     </row>
-    <row r="223" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
         <v>70</v>
       </c>
@@ -3769,7 +3771,7 @@
         <v>36.58</v>
       </c>
     </row>
-    <row r="224" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>70</v>
       </c>
@@ -3783,7 +3785,7 @@
         <v>22.643851017999999</v>
       </c>
     </row>
-    <row r="225" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>70</v>
       </c>
@@ -3797,7 +3799,7 @@
         <v>147.13238000000001</v>
       </c>
     </row>
-    <row r="226" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>70</v>
       </c>
@@ -3811,7 +3813,7 @@
         <v>102.867975</v>
       </c>
     </row>
-    <row r="227" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>70</v>
       </c>
@@ -3825,7 +3827,7 @@
         <v>125.2624716</v>
       </c>
     </row>
-    <row r="228" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
         <v>70</v>
       </c>
@@ -3839,7 +3841,7 @@
         <v>129.71071259999999</v>
       </c>
     </row>
-    <row r="229" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
         <v>70</v>
       </c>
@@ -3853,7 +3855,7 @@
         <v>127.5998</v>
       </c>
     </row>
-    <row r="230" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
         <v>70</v>
       </c>
@@ -3867,7 +3869,7 @@
         <v>466.77496559999997</v>
       </c>
     </row>
-    <row r="231" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>70</v>
       </c>
@@ -3881,7 +3883,7 @@
         <v>270.72160000000002</v>
       </c>
     </row>
-    <row r="232" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
         <v>70</v>
       </c>
@@ -3895,7 +3897,7 @@
         <v>145.33860000000001</v>
       </c>
     </row>
-    <row r="233" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>70</v>
       </c>
@@ -3909,7 +3911,7 @@
         <v>50.883000000000003</v>
       </c>
     </row>
-    <row r="234" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
         <v>70</v>
       </c>
@@ -3923,7 +3925,7 @@
         <v>62.96705</v>
       </c>
     </row>
-    <row r="235" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>70</v>
       </c>
@@ -3937,7 +3939,7 @@
         <v>-33.634174170000001</v>
       </c>
     </row>
-    <row r="236" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
         <v>74</v>
       </c>
@@ -3951,7 +3953,7 @@
         <v>91.021986687999998</v>
       </c>
     </row>
-    <row r="237" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
         <v>74</v>
       </c>
@@ -3965,7 +3967,7 @@
         <v>66.466997524000007</v>
       </c>
     </row>
-    <row r="238" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
         <v>74</v>
       </c>
@@ -3979,7 +3981,7 @@
         <v>41.544733348999998</v>
       </c>
     </row>
-    <row r="239" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
         <v>23</v>
       </c>
@@ -3993,7 +3995,7 @@
         <v>1935.6160052</v>
       </c>
     </row>
-    <row r="240" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
         <v>23</v>
       </c>
@@ -4007,7 +4009,7 @@
         <v>1093.40625</v>
       </c>
     </row>
-    <row r="241" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
         <v>23</v>
       </c>
@@ -4021,7 +4023,7 @@
         <v>936.03599999999994</v>
       </c>
     </row>
-    <row r="242" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
         <v>23</v>
       </c>
@@ -4035,7 +4037,7 @@
         <v>870.293138</v>
       </c>
     </row>
-    <row r="243" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
         <v>23</v>
       </c>
@@ -4049,7 +4051,7 @@
         <v>703.93795499999999</v>
       </c>
     </row>
-    <row r="244" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
         <v>23</v>
       </c>
@@ -4063,7 +4065,7 @@
         <v>453.33</v>
       </c>
     </row>
-    <row r="245" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
         <v>23</v>
       </c>
@@ -4077,7 +4079,7 @@
         <v>490.97399999999999</v>
       </c>
     </row>
-    <row r="246" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
         <v>23</v>
       </c>
@@ -4091,7 +4093,7 @@
         <v>465.35771999999997</v>
       </c>
     </row>
-    <row r="247" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
         <v>23</v>
       </c>
@@ -4105,7 +4107,7 @@
         <v>2569.0349262</v>
       </c>
     </row>
-    <row r="248" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
         <v>23</v>
       </c>
@@ -4119,7 +4121,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="249" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
         <v>23</v>
       </c>
@@ -4133,7 +4135,7 @@
         <v>959.69100000000003</v>
       </c>
     </row>
-    <row r="250" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
         <v>23</v>
       </c>
@@ -4147,7 +4149,7 @@
         <v>284.44299999999998</v>
       </c>
     </row>
-    <row r="251" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
         <v>23</v>
       </c>
@@ -4161,7 +4163,7 @@
         <v>1763.249</v>
       </c>
     </row>
-    <row r="252" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
         <v>23</v>
       </c>
@@ -4175,7 +4177,7 @@
         <v>1752.2063000000001</v>
       </c>
     </row>
-    <row r="253" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
         <v>23</v>
       </c>
@@ -4189,7 +4191,7 @@
         <v>2495.8277849999999</v>
       </c>
     </row>
-    <row r="254" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
         <v>23</v>
       </c>
@@ -4203,7 +4205,7 @@
         <v>2574.3249999999998</v>
       </c>
     </row>
-    <row r="255" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
         <v>23</v>
       </c>
@@ -4217,7 +4219,7 @@
         <v>1101.24</v>
       </c>
     </row>
-    <row r="256" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
         <v>23</v>
       </c>
@@ -4231,7 +4233,7 @@
         <v>191.304</v>
       </c>
     </row>
-    <row r="257" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
         <v>26</v>
       </c>
@@ -4245,7 +4247,7 @@
         <v>388.8</v>
       </c>
     </row>
-    <row r="258" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
         <v>26</v>
       </c>
@@ -4259,7 +4261,7 @@
         <v>106.95099999999999</v>
       </c>
     </row>
-    <row r="259" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
         <v>26</v>
       </c>
@@ -4273,7 +4275,7 @@
         <v>374.26499999999999</v>
       </c>
     </row>
-    <row r="260" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
         <v>26</v>
       </c>
@@ -4287,7 +4289,7 @@
         <v>122.08</v>
       </c>
     </row>
-    <row r="261" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
         <v>26</v>
       </c>
@@ -4301,7 +4303,7 @@
         <v>116.294</v>
       </c>
     </row>
-    <row r="262" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
         <v>26</v>
       </c>
@@ -4315,7 +4317,7 @@
         <v>3805.7429999999999</v>
       </c>
     </row>
-    <row r="263" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
         <v>26</v>
       </c>
@@ -4329,7 +4331,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="264" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
         <v>26</v>
       </c>
@@ -4343,7 +4345,7 @@
         <v>275.238</v>
       </c>
     </row>
-    <row r="265" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
         <v>70</v>
       </c>
@@ -4357,7 +4359,7 @@
         <v>321.96100000000001</v>
       </c>
     </row>
-    <row r="266" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
         <v>70</v>
       </c>
@@ -4371,7 +4373,7 @@
         <v>229.74100000000001</v>
       </c>
     </row>
-    <row r="267" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
         <v>70</v>
       </c>
@@ -4385,7 +4387,7 @@
         <v>157.09299999999999</v>
       </c>
     </row>
-    <row r="268" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
         <v>70</v>
       </c>
@@ -4399,7 +4401,7 @@
         <v>169.16200000000001</v>
       </c>
     </row>
-    <row r="269" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
         <v>70</v>
       </c>
@@ -4413,7 +4415,7 @@
         <v>364.79500000000002</v>
       </c>
     </row>
-    <row r="270" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
         <v>70</v>
       </c>
@@ -4427,7 +4429,7 @@
         <v>28.222999999999999</v>
       </c>
     </row>
-    <row r="271" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
         <v>70</v>
       </c>
@@ -4441,7 +4443,7 @@
         <v>111.91</v>
       </c>
     </row>
-    <row r="272" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
         <v>70</v>
       </c>
@@ -4455,7 +4457,7 @@
         <v>92.884</v>
       </c>
     </row>
-    <row r="273" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
         <v>70</v>
       </c>
@@ -4469,7 +4471,7 @@
         <v>47.414999999999999</v>
       </c>
     </row>
-    <row r="274" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
         <v>70</v>
       </c>
@@ -4483,7 +4485,7 @@
         <v>156.172</v>
       </c>
     </row>
-    <row r="275" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
         <v>18</v>
       </c>
@@ -4494,7 +4496,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="276" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
         <v>18</v>
       </c>
@@ -4508,7 +4510,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="277" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
         <v>18</v>
       </c>
@@ -4522,7 +4524,7 @@
         <v>8.3079999999999998</v>
       </c>
     </row>
-    <row r="278" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
         <v>18</v>
       </c>
@@ -4536,7 +4538,7 @@
         <v>111.676</v>
       </c>
     </row>
-    <row r="279" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
         <v>18</v>
       </c>
@@ -4550,7 +4552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="280" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
         <v>18</v>
       </c>
@@ -4564,7 +4566,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="281" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
         <v>18</v>
       </c>
@@ -4578,7 +4580,7 @@
         <v>66.446399999999997</v>
       </c>
     </row>
-    <row r="282" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
         <v>18</v>
       </c>
@@ -4592,7 +4594,7 @@
         <v>60.198599999999999</v>
       </c>
     </row>
-    <row r="283" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
         <v>18</v>
       </c>
@@ -4606,7 +4608,7 @@
         <v>16.675999999999998</v>
       </c>
     </row>
-    <row r="284" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
         <v>18</v>
       </c>
@@ -4620,7 +4622,7 @@
         <v>16.715</v>
       </c>
     </row>
-    <row r="285" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
         <v>18</v>
       </c>
@@ -4634,7 +4636,7 @@
         <v>38.396999999999998</v>
       </c>
     </row>
-    <row r="286" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
         <v>18</v>
       </c>
@@ -4648,7 +4650,7 @@
         <v>4.25</v>
       </c>
     </row>
-    <row r="287" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
         <v>18</v>
       </c>
@@ -4662,7 +4664,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="288" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
         <v>70</v>
       </c>
@@ -4676,7 +4678,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="289" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
         <v>23</v>
       </c>
@@ -4690,7 +4692,7 @@
         <v>3048</v>
       </c>
     </row>
-    <row r="290" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
         <v>26</v>
       </c>
@@ -4704,7 +4706,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="291" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
         <v>63</v>
       </c>
@@ -4718,7 +4720,7 @@
         <v>74.397000000000006</v>
       </c>
     </row>
-    <row r="292" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
         <v>63</v>
       </c>
@@ -4732,7 +4734,7 @@
         <v>163.31</v>
       </c>
     </row>
-    <row r="293" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
         <v>63</v>
       </c>
@@ -4746,7 +4748,7 @@
         <v>534.41600000000005</v>
       </c>
     </row>
-    <row r="294" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
         <v>63</v>
       </c>
@@ -4760,7 +4762,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="295" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
         <v>50</v>
       </c>
@@ -4774,7 +4776,7 @@
         <v>560.84807000000001</v>
       </c>
     </row>
-    <row r="296" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
         <v>50</v>
       </c>
@@ -4788,7 +4790,7 @@
         <v>480.37799999999999</v>
       </c>
     </row>
-    <row r="297" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
         <v>50</v>
       </c>
@@ -4802,7 +4804,7 @@
         <v>457.70800000000003</v>
       </c>
     </row>
-    <row r="298" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
         <v>50</v>
       </c>
@@ -4816,7 +4818,7 @@
         <v>440.096</v>
       </c>
     </row>
-    <row r="299" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
         <v>50</v>
       </c>
@@ -4830,7 +4832,7 @@
         <v>388.70979</v>
       </c>
     </row>
-    <row r="300" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
         <v>50</v>
       </c>
@@ -4844,7 +4846,7 @@
         <v>386.8227</v>
       </c>
     </row>
-    <row r="301" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
         <v>50</v>
       </c>
@@ -4858,7 +4860,7 @@
         <v>324.61559999999997</v>
       </c>
     </row>
-    <row r="302" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
         <v>50</v>
       </c>
@@ -4872,7 +4874,7 @@
         <v>283.223343</v>
       </c>
     </row>
-    <row r="303" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
         <v>50</v>
       </c>
@@ -4886,7 +4888,7 @@
         <v>257.17744499999998</v>
       </c>
     </row>
-    <row r="304" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
         <v>50</v>
       </c>
@@ -4900,7 +4902,7 @@
         <v>267.80786999999998</v>
       </c>
     </row>
-    <row r="305" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
         <v>50</v>
       </c>
@@ -4914,7 +4916,7 @@
         <v>236.04599999999999</v>
       </c>
     </row>
-    <row r="306" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
         <v>50</v>
       </c>
@@ -4928,7 +4930,7 @@
         <v>207.93639999999999</v>
       </c>
     </row>
-    <row r="307" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
         <v>50</v>
       </c>
@@ -4942,7 +4944,7 @@
         <v>184.02464000000001</v>
       </c>
     </row>
-    <row r="308" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
         <v>50</v>
       </c>
@@ -4956,7 +4958,7 @@
         <v>186.27279999999999</v>
       </c>
     </row>
-    <row r="309" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
         <v>50</v>
       </c>
@@ -4970,7 +4972,7 @@
         <v>181.30464520000001</v>
       </c>
     </row>
-    <row r="310" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
         <v>50</v>
       </c>
@@ -4984,7 +4986,7 @@
         <v>180.90083999999999</v>
       </c>
     </row>
-    <row r="311" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
         <v>50</v>
       </c>
@@ -4998,7 +5000,7 @@
         <v>152.46270000000001</v>
       </c>
     </row>
-    <row r="312" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
         <v>50</v>
       </c>
@@ -5012,7 +5014,7 @@
         <v>152.52197609999999</v>
       </c>
     </row>
-    <row r="313" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
         <v>50</v>
       </c>
@@ -5026,7 +5028,7 @@
         <v>140.721555</v>
       </c>
     </row>
-    <row r="314" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
         <v>50</v>
       </c>
@@ -5040,7 +5042,7 @@
         <v>116.40547100000001</v>
       </c>
     </row>
-    <row r="315" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
         <v>50</v>
       </c>
@@ -5054,7 +5056,7 @@
         <v>115.174015</v>
       </c>
     </row>
-    <row r="316" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
         <v>50</v>
       </c>
@@ -5068,7 +5070,7 @@
         <v>115.07312</v>
       </c>
     </row>
-    <row r="317" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
         <v>50</v>
       </c>
@@ -5082,7 +5084,7 @@
         <v>549.97500000000002</v>
       </c>
     </row>
-    <row r="318" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
         <v>61</v>
       </c>
@@ -5096,7 +5098,7 @@
         <v>455.26299999999998</v>
       </c>
     </row>
-    <row r="319" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
         <v>61</v>
       </c>
@@ -5110,7 +5112,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="320" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
         <v>5</v>
       </c>
@@ -5124,7 +5126,7 @@
         <v>847.84166740000001</v>
       </c>
     </row>
-    <row r="321" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
         <v>5</v>
       </c>
@@ -5138,7 +5140,7 @@
         <v>1503.1095700000001</v>
       </c>
     </row>
-    <row r="322" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
         <v>5</v>
       </c>
@@ -5152,7 +5154,7 @@
         <v>211.977859</v>
       </c>
     </row>
-    <row r="323" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
         <v>5</v>
       </c>
@@ -5166,7 +5168,7 @@
         <v>94.759552999999997</v>
       </c>
     </row>
-    <row r="324" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
         <v>5</v>
       </c>
@@ -5180,7 +5182,7 @@
         <v>487.711995</v>
       </c>
     </row>
-    <row r="325" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
         <v>5</v>
       </c>
@@ -5194,7 +5196,7 @@
         <v>915.09</v>
       </c>
     </row>
-    <row r="326" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
         <v>5</v>
       </c>
@@ -5208,14 +5210,92 @@
         <v>518.94299999999998</v>
       </c>
     </row>
+    <row r="327" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A327" t="s">
+        <v>44</v>
+      </c>
+      <c r="B327" t="s">
+        <v>79</v>
+      </c>
+      <c r="C327" t="s">
+        <v>45</v>
+      </c>
+      <c r="D327">
+        <v>575.76700000000005</v>
+      </c>
+    </row>
+    <row r="328" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A328" t="s">
+        <v>44</v>
+      </c>
+      <c r="B328" t="s">
+        <v>79</v>
+      </c>
+      <c r="C328" t="s">
+        <v>10</v>
+      </c>
+      <c r="D328">
+        <v>145.67400000000001</v>
+      </c>
+    </row>
+    <row r="329" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A329" t="s">
+        <v>44</v>
+      </c>
+      <c r="B329" t="s">
+        <v>79</v>
+      </c>
+      <c r="C329" t="s">
+        <v>49</v>
+      </c>
+      <c r="D329">
+        <v>118.684</v>
+      </c>
+    </row>
+    <row r="330" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A330" t="s">
+        <v>44</v>
+      </c>
+      <c r="B330" t="s">
+        <v>79</v>
+      </c>
+      <c r="C330" t="s">
+        <v>91</v>
+      </c>
+      <c r="D330">
+        <v>104.973</v>
+      </c>
+    </row>
+    <row r="331" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A331" t="s">
+        <v>44</v>
+      </c>
+      <c r="B331" t="s">
+        <v>79</v>
+      </c>
+      <c r="C331" t="s">
+        <v>25</v>
+      </c>
+      <c r="D331">
+        <v>476.053</v>
+      </c>
+    </row>
+    <row r="332" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A332" t="s">
+        <v>44</v>
+      </c>
+      <c r="B332" t="s">
+        <v>79</v>
+      </c>
+      <c r="C332" t="s">
+        <v>40</v>
+      </c>
+      <c r="D332">
+        <v>1165.2354190000001</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E320" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="VCI"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:E326" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>